<commit_message>
Ćw. 7: rozszerzenia (PDF i CSV jako wiedza, eskalacja w agencie, Teams i Slack)
- baza_wiedzy/helpdesk: Regulamin_wsparcia.pdf i Katalog_uslug.csv
  (generator make_wiedza.py, poza zipem), osobne indeksy, żeby nie zmieniać
  wyników SupportAgenta z ćw. 4 i 5
- prompt NorthstarHelpdesk dostosowany do nowych źródeł (REG, KATALOG)
- rozmowy testowe CHAT-09...11, odświeżone arkusze i CSV
- eskalacja w agencie wymaga Action App (Quick Form się nie nadaje)
- wdrożenie na Teams i Slack, uwaga o requesterEmail w czacie
- usunięte zapisy, że agent konwersacyjny jest niedostępny na Community
- zregenerowane HTML, talia i dane; zaktualizowane README, Przewodnik, CLAUDE.md

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UiPath_AI_Warsztat/testy/Northstar_testy.xlsx
+++ b/UiPath_AI_Warsztat/testy/Northstar_testy.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Oczekiwane_wyniki'!$A$1:$K$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Testy_techniczne'!$A$1:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rozmowy_testowe'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rozmowy_testowe'!$A$1:$G$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1482,7 +1482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1795,8 +1795,107 @@
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CHAT-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ewa@example.com</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Ile czasu wsparcie ma na pierwszą odpowiedź przy awarii krytycznej?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A jeśli nikt się do mnie nie odezwie?</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Tura 1: 30 minut w godzinach pracy (REG-2), z zastrzeżeniem, że to czas pierwszej reakcji, a nie naprawy. Tura 2: eskalacja do kierownika wsparcia, kierownik.wsparcia@example.com, z numerem zgłoszenia i nazwą usługi (REG-4); agent sam niczego nie wysyła.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Wiedza z PDF; czas reakcji to nie termin naprawy; rozszerzenie z regulaminem i katalogiem</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>CHAT-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>kasia@example.com</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Kto odpowiada za usługę kadry i jak się z nim skontaktować?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>A kiedy jest tam okno serwisowe?</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Tura 1: Zespół HR Systems, hr-systems@example.com (KATALOG:kadry). Tura 2: sobota 08:00-10:00 (KATALOG:kadry), z pamięcią usługi z tury 1. Bez GetServiceStatus: dla kadry nie ma statusu na żywo.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Wiedza z CSV: wyszukanie wiersza, dokładne wartości; rozszerzenie z regulaminem i katalogiem</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>CHAT-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>bartek@example.com</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Portal nie działa od rana. Kto go prowadzi i kiedy są tam prace serwisowe?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Czyli we wtorek wieczorem to naprawicie?</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Tura 1: GetServiceStatus(portal) -&gt; DEGRADED, bez terminu naprawy (SERVICE:portal); z katalogu Zespół Portal, portal@example.com, okno wtorek 20:00-22:00 (KATALOG:portal). Tura 2: agent nie utożsamia okna serwisowego z terminem naprawy (REG-6); nadal brak potwierdzonego terminu.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Narzędzie i wiedza w jednej odpowiedzi; okno serwisowe to nie termin naprawy; rozszerzenie z regulaminem i katalogiem</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>